<commit_message>
Doku + new License
</commit_message>
<xml_diff>
--- a/time/work_log.xlsx
+++ b/time/work_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\linus\OneDrive\Desktop\Hexapod\time\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\USB Stick\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64D2D7B-4552-489D-AE97-47B3B0B368CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF204B5-89A8-4944-93B1-6D8744D42BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30600" yWindow="-120" windowWidth="30960" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="99">
   <si>
     <t>Work Log</t>
   </si>
@@ -191,104 +191,151 @@
     <t>What was done:</t>
   </si>
   <si>
-    <t>I made a list of ideas, asked my work firends for advice 
-and chose the Hexapod
- Project</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">i made the 
-Hexapod_Themenwahl_250829.pdf, made the github repo and the time plan </t>
+    <t>late</t>
   </si>
   <si>
-    <t xml:space="preserve">i got the approval for
- my Project and in the
- lessons i mostly 
-helped others </t>
+    <t>assambled everything I
+was able to and fixed the
+ordering mistakes</t>
   </si>
   <si>
-    <t xml:space="preserve">got the Büp 
-introduction </t>
+    <t>I was to slow :(</t>
   </si>
   <si>
-    <t>i started with the 3D 
-design and started 
-making first version
- of the leg, and i chose the correct servos</t>
+    <t>I've got the BüP introduction</t>
   </si>
   <si>
-    <t>i finished my prototyp
-and then started on
- makeing a list with
- all the things i want
- to be included in the
- hexapod</t>
+    <t>I made a list of ideas, asked my work friends for advice, and chose the Hexapod project</t>
   </si>
   <si>
-    <t>i started designing 
-the main body and 
-searched all the 
-other components i 
-want to include</t>
+    <t>I created the Hexapod_Themenwahl_250829.pdf file, set up the GitHub repo and developed the time plan.</t>
   </si>
   <si>
-    <t xml:space="preserve">I mostly helped
-others in calss </t>
+    <t>I got the approval for my project, and in the lessons I mostly helped others.</t>
   </si>
   <si>
-    <t>i started to desing the
-main Frame of the
-Hexapod</t>
+    <t>I started with the 3D design and began making the first version of the leg, and I chose the correct servos.</t>
   </si>
   <si>
-    <t>i realised, that the 
-designed mainframe
-wouldent be strong
-enought and i 
-restarted</t>
+    <t>I finished my prototype and then started making a list of all the things I want to be included in the hexapod.</t>
   </si>
   <si>
-    <t>i designed the new
-frame further</t>
+    <t>I started designing the main body and researched all the other components I want to include.</t>
   </si>
   <si>
-    <t>i bought the servos 
-and did organisationl
- stuff</t>
+    <t>I mostly helped others in class.</t>
   </si>
   <si>
-    <t xml:space="preserve">i have started to 
-print the prototype </t>
+    <t>I started to design the main frame of the hexapod.</t>
   </si>
   <si>
-    <t>started with the 
-documentation</t>
+    <t>I realized that the designed mainframe wouldn't be strong enough, and I restarted.</t>
   </si>
   <si>
-    <t xml:space="preserve">finisched the print
- and assambled it and 
-corrected the mistakes </t>
+    <t>I continued designing the new frame</t>
   </si>
   <si>
-    <t xml:space="preserve"> finisched the leg V2 
-and did some 
-organisotional stuff</t>
+    <t>I bought the servos and handled some organizational tasks.</t>
   </si>
   <si>
-    <t>i printed the new 
-leg design and assambled it</t>
+    <t xml:space="preserve">I started to print the prototype </t>
   </si>
   <si>
-    <t>fixed a broken servo
-(not for my project)
-and helped raphael 
-by giving a KiCad 
-course</t>
+    <t>I finished the print, assembled it, and corrected the mistakes.</t>
   </si>
   <si>
-    <t>organisational stuff</t>
+    <t>I started with the documentation.</t>
   </si>
   <si>
-    <t>Finisched 3D design</t>
+    <t>I finished the leg V2 and handled some organizational tasks.</t>
+  </si>
+  <si>
+    <t>I printed the new leg design and assembled it.</t>
+  </si>
+  <si>
+    <t>I fixed a broken servo (not for my project) and helped Raphael by giving a KiCad course.</t>
+  </si>
+  <si>
+    <t>I handled some organizational tasks.</t>
+  </si>
+  <si>
+    <t>I finished the 3D design.</t>
+  </si>
+  <si>
+    <t>I 3D printed the final leg and added the heat-set inserts.</t>
+  </si>
+  <si>
+    <t>I started with the PCB design.</t>
+  </si>
+  <si>
+    <t>I finished the power strip PCBs and searched for parts.</t>
+  </si>
+  <si>
+    <t>I helped Nicola.</t>
+  </si>
+  <si>
+    <t>I started on the mainboard PCB schematic.</t>
+  </si>
+  <si>
+    <t>I continued working on the mainboard PCB schematic.</t>
+  </si>
+  <si>
+    <t>I gave the PCB to Silvano (a PhD student) for review and started on the component layout and PCB edge cuts.</t>
+  </si>
+  <si>
+    <t>I finished the mainboard PCB component layout.</t>
+  </si>
+  <si>
+    <t>I started slicing and printing the rest of the leg parts.</t>
+  </si>
+  <si>
+    <t>I designed the rest of the main body, incorporating the new PCBs.</t>
+  </si>
+  <si>
+    <t>I fixed the issues with the overlapping PCBs in the 3D design and adjusted the shape of the PCBs.</t>
+  </si>
+  <si>
+    <t>I made a commercial render of the mainboard using Blender and several add-ons.</t>
+  </si>
+  <si>
+    <t>I remade the power strip PCB layout, resolved the library issues encountered after switching to Linux (as they weren't saved in the project folder), and purchased the PCB components.</t>
+  </si>
+  <si>
+    <t>I received the PCB schematic review and fixed all the mentioned mistakes.</t>
+  </si>
+  <si>
+    <t>I purchased the new parts that I need.</t>
+  </si>
+  <si>
+    <t>I helped others.</t>
+  </si>
+  <si>
+    <t>I redesigned the mainboard PCB layout.</t>
+  </si>
+  <si>
+    <t>I started printing all of the legs.</t>
+  </si>
+  <si>
+    <t>I continued printing the legs.</t>
+  </si>
+  <si>
+    <t>I finished printing 
+the legs.</t>
+  </si>
+  <si>
+    <t>I assembled the legs.</t>
+  </si>
+  <si>
+    <t>I ordered all of the PCBs from JLCPCB.</t>
+  </si>
+  <si>
+    <t>I searched for the remaining parts and added them to the buy list.</t>
+  </si>
+  <si>
+    <t>I wrote the documentation and started to assemble everything.</t>
   </si>
 </sst>
 </file>
@@ -8005,7 +8052,7 @@
     <row r="2" spans="1:161" x14ac:dyDescent="0.25">
       <c r="A2" s="21">
         <f>COUNTIF(B6:EZ29,TRUE)</f>
-        <v>113</v>
+        <v>271</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="14"/>
@@ -8089,7 +8136,9 @@
       <c r="CC2" s="13"/>
       <c r="CD2" s="13"/>
       <c r="CE2" s="13"/>
-      <c r="CF2" s="13"/>
+      <c r="CF2" s="13" t="s">
+        <v>52</v>
+      </c>
       <c r="CG2" s="13"/>
       <c r="CH2" s="13"/>
       <c r="CI2" s="13"/>
@@ -8110,7 +8159,9 @@
       <c r="CX2" s="13"/>
       <c r="CY2" s="13"/>
       <c r="CZ2" s="13"/>
-      <c r="DA2" s="13"/>
+      <c r="DA2" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="DB2" s="13"/>
       <c r="DC2" s="13"/>
       <c r="DD2" s="13"/>
@@ -8140,7 +8191,7 @@
       <c r="EB2" s="13"/>
       <c r="EC2" s="13"/>
       <c r="ED2" s="36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EE2" s="4" t="s">
         <v>23</v>
@@ -8270,7 +8321,7 @@
       <c r="BW3" s="13"/>
       <c r="BX3" s="13"/>
       <c r="BY3" s="36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BZ3" s="4" t="s">
         <v>20</v>
@@ -8281,7 +8332,7 @@
       <c r="CD3" s="13"/>
       <c r="CE3" s="13"/>
       <c r="CF3" s="36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG3" s="4" t="s">
         <v>21</v>
@@ -12889,7 +12940,7 @@
         <v>0</v>
       </c>
       <c r="CF13" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG13" s="28" t="b">
         <v>0</v>
@@ -13266,7 +13317,7 @@
         <v>0</v>
       </c>
       <c r="AZ14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA14" s="28" t="b">
         <v>0</v>
@@ -13275,10 +13326,10 @@
         <v>0</v>
       </c>
       <c r="BC14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE14" s="28" t="b">
         <v>0</v>
@@ -13287,7 +13338,7 @@
         <v>0</v>
       </c>
       <c r="BG14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH14" s="28" t="b">
         <v>0</v>
@@ -13296,10 +13347,10 @@
         <v>0</v>
       </c>
       <c r="BJ14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL14" s="28" t="b">
         <v>0</v>
@@ -13308,7 +13359,7 @@
         <v>0</v>
       </c>
       <c r="BN14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO14" s="28" t="b">
         <v>0</v>
@@ -13317,10 +13368,10 @@
         <v>0</v>
       </c>
       <c r="BQ14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS14" s="28" t="b">
         <v>0</v>
@@ -13329,7 +13380,7 @@
         <v>0</v>
       </c>
       <c r="BU14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV14" s="28" t="b">
         <v>0</v>
@@ -13338,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="BX14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY14" s="28" t="b">
         <v>0</v>
@@ -13362,7 +13413,7 @@
         <v>0</v>
       </c>
       <c r="CF14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG14" s="28" t="b">
         <v>0</v>
@@ -13380,10 +13431,10 @@
         <v>0</v>
       </c>
       <c r="CL14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN14" s="28" t="b">
         <v>0</v>
@@ -13392,7 +13443,7 @@
         <v>0</v>
       </c>
       <c r="CP14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ14" s="28" t="b">
         <v>0</v>
@@ -13401,7 +13452,7 @@
         <v>0</v>
       </c>
       <c r="CS14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT14" s="28" t="b">
         <v>0</v>
@@ -13413,7 +13464,7 @@
         <v>0</v>
       </c>
       <c r="CW14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX14" s="28" t="b">
         <v>0</v>
@@ -13422,10 +13473,10 @@
         <v>0</v>
       </c>
       <c r="CZ14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DB14" s="28" t="b">
         <v>0</v>
@@ -13443,7 +13494,7 @@
         <v>0</v>
       </c>
       <c r="DG14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH14" s="28" t="b">
         <v>0</v>
@@ -13509,7 +13560,7 @@
         <v>0</v>
       </c>
       <c r="EC14" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED14" s="28" t="b">
         <v>0</v>
@@ -13739,7 +13790,7 @@
         <v>0</v>
       </c>
       <c r="AZ15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA15" s="28" t="b">
         <v>0</v>
@@ -13748,10 +13799,10 @@
         <v>0</v>
       </c>
       <c r="BC15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE15" s="28" t="b">
         <v>0</v>
@@ -13760,7 +13811,7 @@
         <v>0</v>
       </c>
       <c r="BG15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH15" s="28" t="b">
         <v>0</v>
@@ -13769,10 +13820,10 @@
         <v>0</v>
       </c>
       <c r="BJ15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL15" s="28" t="b">
         <v>0</v>
@@ -13781,7 +13832,7 @@
         <v>0</v>
       </c>
       <c r="BN15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO15" s="28" t="b">
         <v>0</v>
@@ -13790,10 +13841,10 @@
         <v>0</v>
       </c>
       <c r="BQ15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS15" s="28" t="b">
         <v>0</v>
@@ -13802,7 +13853,7 @@
         <v>0</v>
       </c>
       <c r="BU15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV15" s="28" t="b">
         <v>0</v>
@@ -13811,7 +13862,7 @@
         <v>0</v>
       </c>
       <c r="BX15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY15" s="28" t="b">
         <v>0</v>
@@ -13835,7 +13886,7 @@
         <v>0</v>
       </c>
       <c r="CF15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG15" s="28" t="b">
         <v>0</v>
@@ -13853,10 +13904,10 @@
         <v>0</v>
       </c>
       <c r="CL15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN15" s="28" t="b">
         <v>0</v>
@@ -13865,7 +13916,7 @@
         <v>0</v>
       </c>
       <c r="CP15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ15" s="28" t="b">
         <v>0</v>
@@ -13874,7 +13925,7 @@
         <v>0</v>
       </c>
       <c r="CS15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT15" s="28" t="b">
         <v>0</v>
@@ -13886,7 +13937,7 @@
         <v>0</v>
       </c>
       <c r="CW15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX15" s="28" t="b">
         <v>0</v>
@@ -13895,10 +13946,10 @@
         <v>0</v>
       </c>
       <c r="CZ15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DB15" s="28" t="b">
         <v>0</v>
@@ -13916,7 +13967,7 @@
         <v>0</v>
       </c>
       <c r="DG15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH15" s="28" t="b">
         <v>0</v>
@@ -13937,7 +13988,7 @@
         <v>0</v>
       </c>
       <c r="DN15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO15" s="28" t="b">
         <v>0</v>
@@ -13982,7 +14033,7 @@
         <v>0</v>
       </c>
       <c r="EC15" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED15" s="28" t="b">
         <v>0</v>
@@ -14212,7 +14263,7 @@
         <v>0</v>
       </c>
       <c r="AZ16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA16" s="28" t="b">
         <v>0</v>
@@ -14221,10 +14272,10 @@
         <v>0</v>
       </c>
       <c r="BC16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE16" s="28" t="b">
         <v>0</v>
@@ -14233,7 +14284,7 @@
         <v>0</v>
       </c>
       <c r="BG16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH16" s="28" t="b">
         <v>0</v>
@@ -14242,10 +14293,10 @@
         <v>0</v>
       </c>
       <c r="BJ16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL16" s="28" t="b">
         <v>0</v>
@@ -14254,7 +14305,7 @@
         <v>0</v>
       </c>
       <c r="BN16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO16" s="28" t="b">
         <v>0</v>
@@ -14263,10 +14314,10 @@
         <v>0</v>
       </c>
       <c r="BQ16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS16" s="28" t="b">
         <v>0</v>
@@ -14275,7 +14326,7 @@
         <v>0</v>
       </c>
       <c r="BU16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV16" s="28" t="b">
         <v>0</v>
@@ -14284,7 +14335,7 @@
         <v>0</v>
       </c>
       <c r="BX16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY16" s="28" t="b">
         <v>0</v>
@@ -14308,7 +14359,7 @@
         <v>0</v>
       </c>
       <c r="CF16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG16" s="28" t="b">
         <v>0</v>
@@ -14326,10 +14377,10 @@
         <v>0</v>
       </c>
       <c r="CL16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN16" s="28" t="b">
         <v>0</v>
@@ -14338,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="CP16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ16" s="28" t="b">
         <v>0</v>
@@ -14347,7 +14398,7 @@
         <v>0</v>
       </c>
       <c r="CS16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT16" s="28" t="b">
         <v>0</v>
@@ -14359,7 +14410,7 @@
         <v>0</v>
       </c>
       <c r="CW16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX16" s="28" t="b">
         <v>0</v>
@@ -14371,7 +14422,7 @@
         <v>0</v>
       </c>
       <c r="DA16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DB16" s="28" t="b">
         <v>0</v>
@@ -14389,7 +14440,7 @@
         <v>0</v>
       </c>
       <c r="DG16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH16" s="28" t="b">
         <v>0</v>
@@ -14410,7 +14461,7 @@
         <v>0</v>
       </c>
       <c r="DN16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO16" s="28" t="b">
         <v>0</v>
@@ -14455,7 +14506,7 @@
         <v>0</v>
       </c>
       <c r="EC16" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED16" s="28" t="b">
         <v>0</v>
@@ -15158,7 +15209,7 @@
         <v>0</v>
       </c>
       <c r="AZ18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA18" s="28" t="b">
         <v>0</v>
@@ -15167,10 +15218,10 @@
         <v>0</v>
       </c>
       <c r="BC18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE18" s="28" t="b">
         <v>0</v>
@@ -15179,7 +15230,7 @@
         <v>0</v>
       </c>
       <c r="BG18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH18" s="28" t="b">
         <v>0</v>
@@ -15188,10 +15239,10 @@
         <v>0</v>
       </c>
       <c r="BJ18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL18" s="28" t="b">
         <v>0</v>
@@ -15200,7 +15251,7 @@
         <v>0</v>
       </c>
       <c r="BN18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO18" s="28" t="b">
         <v>0</v>
@@ -15209,10 +15260,10 @@
         <v>0</v>
       </c>
       <c r="BQ18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS18" s="28" t="b">
         <v>0</v>
@@ -15221,7 +15272,7 @@
         <v>0</v>
       </c>
       <c r="BU18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV18" s="28" t="b">
         <v>0</v>
@@ -15230,7 +15281,7 @@
         <v>0</v>
       </c>
       <c r="BX18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY18" s="28" t="b">
         <v>0</v>
@@ -15254,7 +15305,7 @@
         <v>0</v>
       </c>
       <c r="CF18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG18" s="28" t="b">
         <v>0</v>
@@ -15272,10 +15323,10 @@
         <v>0</v>
       </c>
       <c r="CL18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN18" s="28" t="b">
         <v>0</v>
@@ -15284,7 +15335,7 @@
         <v>0</v>
       </c>
       <c r="CP18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ18" s="28" t="b">
         <v>0</v>
@@ -15293,7 +15344,7 @@
         <v>0</v>
       </c>
       <c r="CS18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT18" s="28" t="b">
         <v>0</v>
@@ -15305,7 +15356,7 @@
         <v>0</v>
       </c>
       <c r="CW18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX18" s="28" t="b">
         <v>0</v>
@@ -15314,7 +15365,7 @@
         <v>0</v>
       </c>
       <c r="CZ18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA18" s="28" t="b">
         <v>0</v>
@@ -15335,7 +15386,7 @@
         <v>0</v>
       </c>
       <c r="DG18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH18" s="28" t="b">
         <v>0</v>
@@ -15347,7 +15398,7 @@
         <v>0</v>
       </c>
       <c r="DK18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL18" s="28" t="b">
         <v>0</v>
@@ -15356,7 +15407,7 @@
         <v>0</v>
       </c>
       <c r="DN18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO18" s="28" t="b">
         <v>0</v>
@@ -15401,7 +15452,7 @@
         <v>0</v>
       </c>
       <c r="EC18" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED18" s="28" t="b">
         <v>0</v>
@@ -15631,7 +15682,7 @@
         <v>0</v>
       </c>
       <c r="AZ19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA19" s="28" t="b">
         <v>0</v>
@@ -15640,10 +15691,10 @@
         <v>0</v>
       </c>
       <c r="BC19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE19" s="28" t="b">
         <v>0</v>
@@ -15652,7 +15703,7 @@
         <v>0</v>
       </c>
       <c r="BG19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH19" s="28" t="b">
         <v>0</v>
@@ -15661,10 +15712,10 @@
         <v>0</v>
       </c>
       <c r="BJ19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL19" s="28" t="b">
         <v>0</v>
@@ -15673,7 +15724,7 @@
         <v>0</v>
       </c>
       <c r="BN19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO19" s="28" t="b">
         <v>0</v>
@@ -15682,10 +15733,10 @@
         <v>0</v>
       </c>
       <c r="BQ19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS19" s="28" t="b">
         <v>0</v>
@@ -15694,7 +15745,7 @@
         <v>0</v>
       </c>
       <c r="BU19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV19" s="28" t="b">
         <v>0</v>
@@ -15703,7 +15754,7 @@
         <v>0</v>
       </c>
       <c r="BX19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY19" s="28" t="b">
         <v>0</v>
@@ -15727,7 +15778,7 @@
         <v>0</v>
       </c>
       <c r="CF19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG19" s="28" t="b">
         <v>0</v>
@@ -15745,10 +15796,10 @@
         <v>0</v>
       </c>
       <c r="CL19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN19" s="28" t="b">
         <v>0</v>
@@ -15757,7 +15808,7 @@
         <v>0</v>
       </c>
       <c r="CP19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ19" s="28" t="b">
         <v>0</v>
@@ -15766,7 +15817,7 @@
         <v>0</v>
       </c>
       <c r="CS19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT19" s="28" t="b">
         <v>0</v>
@@ -15778,7 +15829,7 @@
         <v>0</v>
       </c>
       <c r="CW19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX19" s="28" t="b">
         <v>0</v>
@@ -15787,7 +15838,7 @@
         <v>0</v>
       </c>
       <c r="CZ19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA19" s="28" t="b">
         <v>0</v>
@@ -15808,7 +15859,7 @@
         <v>0</v>
       </c>
       <c r="DG19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH19" s="28" t="b">
         <v>0</v>
@@ -15820,7 +15871,7 @@
         <v>0</v>
       </c>
       <c r="DK19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL19" s="28" t="b">
         <v>0</v>
@@ -15829,7 +15880,7 @@
         <v>0</v>
       </c>
       <c r="DN19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO19" s="28" t="b">
         <v>0</v>
@@ -15874,7 +15925,7 @@
         <v>0</v>
       </c>
       <c r="EC19" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED19" s="28" t="b">
         <v>0</v>
@@ -16104,7 +16155,7 @@
         <v>0</v>
       </c>
       <c r="AZ20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA20" s="28" t="b">
         <v>0</v>
@@ -16113,10 +16164,10 @@
         <v>0</v>
       </c>
       <c r="BC20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE20" s="28" t="b">
         <v>0</v>
@@ -16125,7 +16176,7 @@
         <v>0</v>
       </c>
       <c r="BG20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH20" s="28" t="b">
         <v>0</v>
@@ -16137,7 +16188,7 @@
         <v>0</v>
       </c>
       <c r="BK20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BL20" s="28" t="b">
         <v>0</v>
@@ -16146,7 +16197,7 @@
         <v>0</v>
       </c>
       <c r="BN20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO20" s="28" t="b">
         <v>0</v>
@@ -16155,10 +16206,10 @@
         <v>0</v>
       </c>
       <c r="BQ20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS20" s="28" t="b">
         <v>0</v>
@@ -16167,7 +16218,7 @@
         <v>0</v>
       </c>
       <c r="BU20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV20" s="28" t="b">
         <v>0</v>
@@ -16176,7 +16227,7 @@
         <v>0</v>
       </c>
       <c r="BX20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY20" s="28" t="b">
         <v>0</v>
@@ -16218,10 +16269,10 @@
         <v>0</v>
       </c>
       <c r="CL20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN20" s="28" t="b">
         <v>0</v>
@@ -16230,7 +16281,7 @@
         <v>0</v>
       </c>
       <c r="CP20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ20" s="28" t="b">
         <v>0</v>
@@ -16239,7 +16290,7 @@
         <v>0</v>
       </c>
       <c r="CS20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT20" s="28" t="b">
         <v>0</v>
@@ -16251,7 +16302,7 @@
         <v>0</v>
       </c>
       <c r="CW20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX20" s="28" t="b">
         <v>0</v>
@@ -16260,7 +16311,7 @@
         <v>0</v>
       </c>
       <c r="CZ20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA20" s="28" t="b">
         <v>0</v>
@@ -16281,7 +16332,7 @@
         <v>0</v>
       </c>
       <c r="DG20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DH20" s="28" t="b">
         <v>0</v>
@@ -16293,7 +16344,7 @@
         <v>0</v>
       </c>
       <c r="DK20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL20" s="28" t="b">
         <v>0</v>
@@ -16302,7 +16353,7 @@
         <v>0</v>
       </c>
       <c r="DN20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO20" s="28" t="b">
         <v>0</v>
@@ -16347,7 +16398,7 @@
         <v>0</v>
       </c>
       <c r="EC20" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED20" s="28" t="b">
         <v>0</v>
@@ -16577,7 +16628,7 @@
         <v>0</v>
       </c>
       <c r="AZ21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BA21" s="28" t="b">
         <v>0</v>
@@ -16586,10 +16637,10 @@
         <v>0</v>
       </c>
       <c r="BC21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE21" s="28" t="b">
         <v>0</v>
@@ -16598,7 +16649,7 @@
         <v>0</v>
       </c>
       <c r="BG21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH21" s="28" t="b">
         <v>0</v>
@@ -16619,7 +16670,7 @@
         <v>0</v>
       </c>
       <c r="BN21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO21" s="28" t="b">
         <v>0</v>
@@ -16628,10 +16679,10 @@
         <v>0</v>
       </c>
       <c r="BQ21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS21" s="28" t="b">
         <v>0</v>
@@ -16640,7 +16691,7 @@
         <v>0</v>
       </c>
       <c r="BU21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV21" s="28" t="b">
         <v>0</v>
@@ -16649,7 +16700,7 @@
         <v>0</v>
       </c>
       <c r="BX21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BY21" s="28" t="b">
         <v>0</v>
@@ -16691,10 +16742,10 @@
         <v>0</v>
       </c>
       <c r="CL21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN21" s="28" t="b">
         <v>0</v>
@@ -16703,7 +16754,7 @@
         <v>0</v>
       </c>
       <c r="CP21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ21" s="28" t="b">
         <v>0</v>
@@ -16712,7 +16763,7 @@
         <v>0</v>
       </c>
       <c r="CS21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT21" s="28" t="b">
         <v>0</v>
@@ -16724,7 +16775,7 @@
         <v>0</v>
       </c>
       <c r="CW21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX21" s="28" t="b">
         <v>0</v>
@@ -16733,7 +16784,7 @@
         <v>0</v>
       </c>
       <c r="CZ21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA21" s="28" t="b">
         <v>0</v>
@@ -16766,7 +16817,7 @@
         <v>0</v>
       </c>
       <c r="DK21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL21" s="28" t="b">
         <v>0</v>
@@ -16820,7 +16871,7 @@
         <v>0</v>
       </c>
       <c r="EC21" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED21" s="28" t="b">
         <v>0</v>
@@ -17062,7 +17113,7 @@
         <v>0</v>
       </c>
       <c r="BD22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE22" s="28" t="b">
         <v>0</v>
@@ -17092,7 +17143,7 @@
         <v>0</v>
       </c>
       <c r="BN22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO22" s="28" t="b">
         <v>0</v>
@@ -17101,7 +17152,7 @@
         <v>0</v>
       </c>
       <c r="BQ22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR22" s="28" t="b">
         <v>0</v>
@@ -17164,10 +17215,10 @@
         <v>0</v>
       </c>
       <c r="CL22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CN22" s="28" t="b">
         <v>0</v>
@@ -17185,7 +17236,7 @@
         <v>0</v>
       </c>
       <c r="CS22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CT22" s="28" t="b">
         <v>0</v>
@@ -17197,7 +17248,7 @@
         <v>0</v>
       </c>
       <c r="CW22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CX22" s="28" t="b">
         <v>0</v>
@@ -17206,7 +17257,7 @@
         <v>0</v>
       </c>
       <c r="CZ22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA22" s="28" t="b">
         <v>0</v>
@@ -17239,7 +17290,7 @@
         <v>0</v>
       </c>
       <c r="DK22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL22" s="28" t="b">
         <v>0</v>
@@ -17293,7 +17344,7 @@
         <v>0</v>
       </c>
       <c r="EC22" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ED22" s="28" t="b">
         <v>0</v>
@@ -17721,7 +17772,7 @@
         <v>0</v>
       </c>
       <c r="DN23" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO23" s="28" t="b">
         <v>0</v>
@@ -18194,7 +18245,7 @@
         <v>0</v>
       </c>
       <c r="DN24" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DO24" s="28" t="b">
         <v>0</v>
@@ -20680,84 +20731,84 @@
       </c>
     </row>
     <row r="30" spans="1:157" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:157" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:157" ht="150.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B31" s="37" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H31" s="16"/>
       <c r="I31" s="16" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J31" s="16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K31" s="15"/>
       <c r="L31" s="15"/>
       <c r="M31" s="16" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="N31" s="16" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="O31" s="15"/>
       <c r="P31" s="16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="Q31" s="16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="R31" s="15"/>
       <c r="S31" s="15"/>
       <c r="T31" s="16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="U31" s="16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="V31" s="15"/>
       <c r="W31" s="15"/>
       <c r="X31" s="16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="Y31" s="15"/>
       <c r="Z31" s="15"/>
       <c r="AA31" s="16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AB31" s="16" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="AC31" s="15"/>
       <c r="AD31" s="15"/>
       <c r="AE31" s="16" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="AF31" s="15"/>
       <c r="AG31" s="15"/>
       <c r="AH31" s="16" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AI31" s="16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="AJ31" s="15"/>
       <c r="AK31" s="16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AL31" s="15" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AM31" s="15"/>
       <c r="AN31" s="15"/>
@@ -20771,76 +20822,130 @@
       <c r="AV31" s="15"/>
       <c r="AW31" s="15"/>
       <c r="AX31" s="15" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="AY31" s="15"/>
-      <c r="AZ31" s="15"/>
+      <c r="AZ31" s="16" t="s">
+        <v>75</v>
+      </c>
       <c r="BA31" s="15"/>
       <c r="BB31" s="15"/>
-      <c r="BC31" s="15"/>
-      <c r="BD31" s="15"/>
+      <c r="BC31" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="BD31" s="16" t="s">
+        <v>77</v>
+      </c>
       <c r="BE31" s="15"/>
-      <c r="BF31" s="15"/>
-      <c r="BG31" s="15"/>
+      <c r="BF31" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="BG31" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="BH31" s="15"/>
       <c r="BI31" s="15"/>
-      <c r="BJ31" s="15"/>
-      <c r="BK31" s="15"/>
+      <c r="BJ31" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="BK31" s="16" t="s">
+        <v>81</v>
+      </c>
       <c r="BL31" s="15"/>
       <c r="BM31" s="15"/>
-      <c r="BN31" s="15"/>
+      <c r="BN31" s="16" t="s">
+        <v>82</v>
+      </c>
       <c r="BO31" s="15"/>
       <c r="BP31" s="15"/>
-      <c r="BQ31" s="15"/>
-      <c r="BR31" s="15"/>
+      <c r="BQ31" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="BR31" s="16" t="s">
+        <v>84</v>
+      </c>
       <c r="BS31" s="15"/>
       <c r="BT31" s="15"/>
-      <c r="BU31" s="15"/>
+      <c r="BU31" s="16" t="s">
+        <v>85</v>
+      </c>
       <c r="BV31" s="15"/>
       <c r="BW31" s="15"/>
-      <c r="BX31" s="15"/>
-      <c r="BY31" s="15"/>
+      <c r="BX31" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="BY31" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="BZ31" s="15"/>
       <c r="CA31" s="15"/>
       <c r="CB31" s="15"/>
       <c r="CC31" s="15"/>
       <c r="CD31" s="15"/>
       <c r="CE31" s="15"/>
-      <c r="CF31" s="15"/>
+      <c r="CF31" s="16" t="s">
+        <v>87</v>
+      </c>
       <c r="CG31" s="15"/>
       <c r="CH31" s="15"/>
       <c r="CI31" s="15"/>
       <c r="CJ31" s="15"/>
       <c r="CK31" s="15"/>
-      <c r="CL31" s="15"/>
-      <c r="CM31" s="15"/>
+      <c r="CL31" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM31" s="16" t="s">
+        <v>89</v>
+      </c>
       <c r="CN31" s="15"/>
-      <c r="CO31" s="15"/>
-      <c r="CP31" s="15"/>
+      <c r="CO31" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="CP31" s="16" t="s">
+        <v>91</v>
+      </c>
       <c r="CQ31" s="15"/>
       <c r="CR31" s="15"/>
-      <c r="CS31" s="15"/>
+      <c r="CS31" s="16" t="s">
+        <v>92</v>
+      </c>
       <c r="CT31" s="15"/>
       <c r="CU31" s="15"/>
       <c r="CV31" s="15"/>
-      <c r="CW31" s="15"/>
+      <c r="CW31" s="16" t="s">
+        <v>93</v>
+      </c>
       <c r="CX31" s="15"/>
       <c r="CY31" s="15"/>
-      <c r="CZ31" s="15"/>
-      <c r="DA31" s="15"/>
+      <c r="CZ31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="DA31" s="15" t="s">
+        <v>95</v>
+      </c>
       <c r="DB31" s="15"/>
-      <c r="DC31" s="15"/>
+      <c r="DC31" s="15" t="s">
+        <v>90</v>
+      </c>
       <c r="DD31" s="15"/>
       <c r="DE31" s="15"/>
       <c r="DF31" s="15"/>
-      <c r="DG31" s="15"/>
+      <c r="DG31" s="16" t="s">
+        <v>96</v>
+      </c>
       <c r="DH31" s="15"/>
       <c r="DI31" s="15"/>
-      <c r="DJ31" s="15"/>
-      <c r="DK31" s="15"/>
+      <c r="DJ31" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="DK31" s="16" t="s">
+        <v>97</v>
+      </c>
       <c r="DL31" s="15"/>
       <c r="DM31" s="15"/>
-      <c r="DN31" s="15"/>
+      <c r="DN31" s="16" t="s">
+        <v>98</v>
+      </c>
       <c r="DO31" s="15"/>
       <c r="DP31" s="15"/>
       <c r="DQ31" s="15"/>
@@ -20855,7 +20960,9 @@
       <c r="DZ31" s="15"/>
       <c r="EA31" s="15"/>
       <c r="EB31" s="15"/>
-      <c r="EC31" s="15"/>
+      <c r="EC31" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="ED31" s="15"/>
       <c r="EE31" s="15"/>
       <c r="EF31" s="15"/>

</xml_diff>